<commit_message>
results: Canada scenario set, priority-1 runs (nine runs on base v6f) + analysis script
Nine Canada scenario runs (c01a gridmix, c02a localcontent, c03b nuclear_se,
c04a partnership, c06b dcpipeline, c07a windpaced, c07b windaccel, c08b minerals,
c09a euprojects), all OPTIMAL with infeasibility-slack generation equal to the base.
Write-up with per-year tables, scenario notes, the scenario-5 side calculation and
the implementation record; plan workbook gets an Implemented_p1 sheet; scenario
mapping extended; Scripts/analyze_canada.py (table, markdown, per-run gate).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/proposals/CA_scenario_plan_2026-10-04.xlsx
+++ b/docs/proposals/CA_scenario_plan_2026-10-04.xlsx
@@ -17,6 +17,7 @@
     <sheet name="Model baseline" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="CER comparison" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Open questions" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Implemented_p1" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Overview'!$A$1:$M$10</definedName>
@@ -26,6 +27,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Run plan'!$A$1:$G$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Sources'!$A$1:$F$144</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Open questions'!$A$1:$D$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Implemented_p1'!$A$1:$H$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -553,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -569,7 +571,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Prepared 2026-10-05 for the nine Canada scenarios requested by Siemens Energy Canada (docs/proposals/canada.txt). Status: PLAN - nothing is implemented or run. Numbers come from web-sourced reports (2025-2026 vintage, research notes A-E in this folder) plus the model baseline; every number in "Assumptions" carries a source id or is explicitly marked as an assumption.</t>
+          <t>Prepared 2026-10-06 for the nine Canada scenarios requested by Siemens Energy Canada (docs/proposals/canada.txt). Status: PLAN - nothing is implemented or run. Numbers come from web-sourced reports (2025-2026 vintage, research notes A-E in this folder) plus the model baseline; every number in "Assumptions" carries a source id or is explicitly marked as an assumption.</t>
         </is>
       </c>
     </row>
@@ -654,31 +656,38 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Implemented_p1 - implementation record of the priority-1 runs (2026-10-05/06): data folder, definition as implemented, deviation from the plan, status, headline result. Results: scenario_plan_canada_2026-10-04/RESULTS_canada_p1_2026-10-06.md</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
         <is>
           <t>Conventions</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Canada is one model node (no provinces, no territories, no off-grid systems). Years 2025-2040 annual; 2050 targets enter through their 2040 waypoint. Demand in busbar TWh. Costs in EUR2023 (1 USD = 0.925 EUR; 1 CAD = 0.685 EUR). Capacity in GW.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Effort: S = data rows via the existing scenario generator (&lt; 1 day incl. run); M = new lever or new technology rows (1-3 days); L = model change or external dependency.</t>
+          <t>Canada is one model node (no provinces, no territories, no off-grid systems). Years 2025-2040 annual; 2050 targets enter through their 2040 waypoint. Demand in busbar TWh. Costs in EUR2023 (1 USD = 0.925 EUR; 1 CAD = 0.685 EUR). Capacity in GW.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Effort: S = data rows via the existing scenario generator (&lt; 1 day incl. run); M = new lever or new technology rows (1-3 days); L = model change or external dependency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Tags from the request: [Tailwind] upside to load / SE market, [Headwind] downside, [Mixed].</t>
         </is>
@@ -948,6 +957,493 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:D12"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="90" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Run label</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Variant</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Data folder</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>As implemented</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Deviation from the plan</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Canada 2040 headline (vs base)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>fel2026_c01a_gridmix_49_2015_v6</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>1A</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>NorthAmerica_c01a_gridmix</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>New-CCGT minimum 8.6 / 14.5 / 24.5 GW (2030 / 2035 / 2040) so that the gas fleet follows CER Current Measures 34.2 / 33.4 / 36.6 GW; SMR 0.3 / 1.5 / 2.1 GW (min = max); batteries 4.5 / 6.5 / 10.5 GW minimum.</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>In 2027-28 the base corridor ceiling binds; the minimum is held 0.1 % under it.</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>OPTIMAL, slack = base</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>gas +9.4 GW, wind -20.9 GW, CO2 +15.5 Mt, cost +6.4 bEUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>fel2026_c02a_localcontent_49_2015_v6</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>2A</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>NorthAmerica_c02a_localcontent</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Canada capital cost from 2028: onshore wind x1.08, utility PV x1.06, Li-ion x1.06 (power and energy component), CCGT x1.05; written for every year of the World cost rows.</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>OPTIMAL, slack = base</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>wind build shifted 2032-35 -&gt; 2037-39; 2040 wind -2.5 GW; cost +2.0 bEUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>fel2026_c03b_nuclear_se_49_2015_v6</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>3B</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>NorthAmerica_c03b_nuclear_se</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Canada rows of the existing nuclear_announced overlay: large reactors 11.5 / 15.6 / 17.9 / 23.4 GW (2030 / 2035 / 2038 / 2040), SMR 0.6 / 1.8 / 3.0 / 4.2 GW as minima (SMR ceiling = minimum + 1 MW).</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>OPTIMAL, slack = base</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>nuclear +11.7 GW, wind -22 GW, exports +7 TWh, cost +8.9 bEUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>fel2026_c04a_partnership_49_2015_v6</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>4A</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>NorthAmerica_c04a_partnership</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Capital-cost factors from the annuity ratio CRF(4.83 %) / CRF(5 %) with the lifetimes of the data: wind 0.982, utility PV 0.979, hydro 0.972, nuclear 0.971 (2026-2040); wind and PV ceiling one year earlier; hydro and nuclear minimum and maximum two years earlier.</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>OPTIMAL, slack = base</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>solar +5.3 GW, gas -4 TWh, cost +0.1 bEUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>(side calculation)</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>S5</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>5A / 5B</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Table in RESULTS_canada_p1_2026-10-06.md (demand +0.9 / +2.5 TWh, diesel displaced 0.8 / 1.2 TWh, hydro +0.09 / +0.10 GW, microreactors 0.02 / 0.05 GW by 2040).</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>as planned</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>0.1-0.3 % of the Canada node</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>fel2026_c06b_dcpipeline_49_2015_v6</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>6B</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>NorthAmerica_c06b_dcpipeline</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Power_DataCenter Canada 47 / 121 / 177 TWh (2030 / 2035 / 2040), linear from the base 2025 value; gas minimum unchanged (dedicated gas inside the forced CCGT).</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>OPTIMAL, slack = base</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>demand -92 TWh, wind -25.4 GW, exports +10 TWh, cost -14.6 bEUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>fel2026_c07a_windpaced_49_2015_v6</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>S7</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>7A</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>NorthAmerica_c07a_windpaced</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Group ceiling Onshore x Canada 28.0 / 43.5 / 55.7 GW (linear from the 2025 fleet); wind minimum lowered to the ceiling in 2030-2036; onshore wind capital cost x1.13 from 2026.</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>OPTIMAL, slack = base</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>wind -31.5 GW, gas +9.3 GW / +78 TWh, CO2 +26.4 Mt, cost +3.8 bEUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>fel2026_c07b_windaccel_49_2015_v6</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>S7</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>7B</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>NorthAmerica_c07b_windaccel</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Wind (average class) minimum: base corridor to 2027, then linear to 45 (2030) / 70 (2035) / 87 GW (2040); ceiling lifted to the floor +2 % in 2028-2030; capital cost x0.948 / 0.93 / 0.91 (2030 / 2035 / 2040, interpolated from 1.0 in 2025).</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Floor starts from the 2027 corridor value instead of 2025 (projects under construction are known).</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>OPTIMAL, slack = base</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>wind +11.0 GW (98 GW total: better class added on top of the floor), gas -15 TWh, cost -1.2 bEUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>fel2026_c08b_minerals_49_2015_v6</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>S8</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>8B</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>NorthAmerica_c08b_minerals</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Power_LargeLoads Canada +7.5 / +19.7 / +21.7 TWh (2030 / 2035 / 2040), flat profile, linear from zero in 2025; own filter file (fuel Power_LargeLoads, mode 7).</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>OPTIMAL, slack = base</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>wind +6.6 GW, cost +4.5 bEUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>fel2026_c09a_euprojects_49_2015_v6</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>S9</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>9A</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>NorthAmerica_c09a_euprojects</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Power_Hydrogen Canada +4 / +26 / +36 TWh and Power_LargeLoads +8 / +19 / +29 TWh (2030 / 2035 / 2040) on top of the base, linear from zero in 2025.</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>OPTIMAL, slack = base</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>wind +18.9 GW, exports -7 TWh, cost +10.4 bEUR</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>